<commit_message>
fix(qa): ensure robust JSON parsing of test results and genuine pass status tracking
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Selenium_Failed_Tests.xlsx
+++ b/Test Results/Excel/Selenium_Failed_Tests.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="99">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -62,13 +62,281 @@
   </si>
   <si>
     <t>GitHub Run Number</t>
+  </si>
+  <si>
+    <t>TC_WEB_AUTH_001</t>
+  </si>
+  <si>
+    <t>Authentication</t>
+  </si>
+  <si>
+    <t>Web login with valid student credentials - Case 1</t>
+  </si>
+  <si>
+    <t>Verify that a student can successfully log in on web layout. (Variation 1)</t>
+  </si>
+  <si>
+    <t>HIGH</t>
+  </si>
+  <si>
+    <t>Student account exists.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Launch browser.
+2. Navigate to BASE_URL.
+3. Enter valid student email.
+4. Enter valid student password.
+5. Click Login button.</t>
+  </si>
+  <si>
+    <t>email: "student@college.edu", password: "student123"</t>
+  </si>
+  <si>
+    <t>User is successfully logged in and redirected to web Student Dashboard.</t>
+  </si>
+  <si>
+    <t>Web element selection failure / validation assertion failed.</t>
+  </si>
+  <si>
+    <t>FAILED</t>
+  </si>
+  <si>
+    <t>5.35s</t>
+  </si>
+  <si>
+    <t>expected false to be true</t>
+  </si>
+  <si>
+    <t>automation/selenium/screenshots/TC_WEB_AUTH_001_failed.png</t>
+  </si>
+  <si>
+    <t>automation/selenium/logs/browser-console.log</t>
+  </si>
+  <si>
+    <t>smoke.web.test.ts</t>
+  </si>
+  <si>
+    <t>LOCAL</t>
+  </si>
+  <si>
+    <t>TC_WEB_AUTH_002</t>
+  </si>
+  <si>
+    <t>Web login empty fields verification - Case 2</t>
+  </si>
+  <si>
+    <t>Verify validation messages show when submitting blank credentials. (Variation 2)</t>
+  </si>
+  <si>
+    <t>MEDIUM</t>
+  </si>
+  <si>
+    <t>None.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Navigate to login form.
+2. Leave fields blank.
+3. Click Login.</t>
+  </si>
+  <si>
+    <t>Validation markers light up on blank text-inputs.</t>
+  </si>
+  <si>
+    <t>15.05s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, [data-testid="login_email"], input[type="email"])
+Wait timed out after 15051ms</t>
+  </si>
+  <si>
+    <t>automation/selenium/screenshots/TC_WEB_AUTH_002_failed.png</t>
+  </si>
+  <si>
+    <t>TC_WEB_AUTH_003</t>
+  </si>
+  <si>
+    <t>Web login with valid student credentials - Case 3</t>
+  </si>
+  <si>
+    <t>Verify that a student can successfully log in on web layout. (Variation 3)</t>
+  </si>
+  <si>
+    <t>15.11s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, [data-testid="login_email"], input[type="email"])
+Wait timed out after 15105ms</t>
+  </si>
+  <si>
+    <t>automation/selenium/screenshots/TC_WEB_AUTH_003_failed.png</t>
+  </si>
+  <si>
+    <t>TC_WEB_NAV_001</t>
+  </si>
+  <si>
+    <t>Navigation</t>
+  </si>
+  <si>
+    <t>Click header back button in details page - Case 1</t>
+  </si>
+  <si>
+    <t>Verify user is returned to the correct scroll index on feed. (Variation 1)</t>
+  </si>
+  <si>
+    <t>Event detail page is open.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Click Back button in details modal.
+2. Verify current view.</t>
+  </si>
+  <si>
+    <t>Details panel is closed, feed listing state remains untouched.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, [data-testid^="event_card_"], div[role="button"])
+Wait timed out after 15054ms</t>
+  </si>
+  <si>
+    <t>automation/selenium/screenshots/TC_WEB_NAV_001_failed.png</t>
+  </si>
+  <si>
+    <t>TC_WEB_NAV_002</t>
+  </si>
+  <si>
+    <t>Click header back button in details page - Case 2</t>
+  </si>
+  <si>
+    <t>Verify user is returned to the correct scroll index on feed. (Variation 2)</t>
+  </si>
+  <si>
+    <t>15.07s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, [data-testid="tab_profile"])
+Wait timed out after 15070ms</t>
+  </si>
+  <si>
+    <t>automation/selenium/screenshots/TC_WEB_NAV_002_failed.png</t>
+  </si>
+  <si>
+    <t>TC_WEB_FORM_001</t>
+  </si>
+  <si>
+    <t>Forms</t>
+  </si>
+  <si>
+    <t>Fill event creation details - Case 1</t>
+  </si>
+  <si>
+    <t>Verify event inputs function. (Variation 1)</t>
+  </si>
+  <si>
+    <t>Create Form open.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Fill Title.
+2. Select Datepicker.
+3. Enter Desc.
+4. Click Create.</t>
+  </si>
+  <si>
+    <t>title: "Web Tech Meet"</t>
+  </si>
+  <si>
+    <t>Input fields contain typed strings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, [data-testid="profile_edit"])
+Wait timed out after 15065ms</t>
+  </si>
+  <si>
+    <t>automation/selenium/screenshots/TC_WEB_FORM_001_failed.png</t>
+  </si>
+  <si>
+    <t>TC_WEB_CRUD_001</t>
+  </si>
+  <si>
+    <t>CRUD</t>
+  </si>
+  <si>
+    <t>Student registration for event on web client - Case 1</t>
+  </si>
+  <si>
+    <t>Verify registering updates status on database. (Variation 1)</t>
+  </si>
+  <si>
+    <t>User is logged in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Select active event.
+2. Click Register.
+3. Confirm dialog.
+4. Check button status.</t>
+  </si>
+  <si>
+    <t>event_id: "607d2c33"</t>
+  </si>
+  <si>
+    <t>Status changes to Cancel Registration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, [data-testid="dashboard_search"], input[placeholder*="Search"])
+Wait timed out after 15110ms</t>
+  </si>
+  <si>
+    <t>automation/selenium/screenshots/TC_WEB_CRUD_001_failed.png</t>
+  </si>
+  <si>
+    <t>TC_WEB_CRUD_003</t>
+  </si>
+  <si>
+    <t>Student registration for event on web client - Case 3</t>
+  </si>
+  <si>
+    <t>Verify registering updates status on database. (Variation 3)</t>
+  </si>
+  <si>
+    <t>15.03s</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting for element to be located By(css selector, [data-testid="event_detail_back"])
+Wait timed out after 15023ms</t>
+  </si>
+  <si>
+    <t>automation/selenium/screenshots/TC_WEB_CRUD_003_failed.png</t>
+  </si>
+  <si>
+    <t>TC_WEB_SESS_001</t>
+  </si>
+  <si>
+    <t>Session Management</t>
+  </si>
+  <si>
+    <t>Verify session persistence across reload - Case 1</t>
+  </si>
+  <si>
+    <t>Verify token remains in localStorage on refresh. (Variation 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Verify homepage dashboard.
+2. Reload page.
+3. Inspect current view.</t>
+  </si>
+  <si>
+    <t>Dashboard continues loading direct, bypassing login screen.</t>
+  </si>
+  <si>
+    <t>5.08s</t>
+  </si>
+  <si>
+    <t>automation/selenium/screenshots/TC_WEB_SESS_001_failed.png</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -80,8 +348,12 @@
       <b/>
       <color rgb="FFFFFF"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="C65911"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -91,6 +363,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,9 +383,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -448,7 +726,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -520,6 +798,483 @@
         <v>16</v>
       </c>
     </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" t="s">
+        <v>25</v>
+      </c>
+      <c r="J2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L2" t="s">
+        <v>28</v>
+      </c>
+      <c r="M2" t="s">
+        <v>29</v>
+      </c>
+      <c r="N2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O2" t="s">
+        <v>31</v>
+      </c>
+      <c r="P2" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" t="s">
+        <v>41</v>
+      </c>
+      <c r="M3" t="s">
+        <v>42</v>
+      </c>
+      <c r="N3" t="s">
+        <v>43</v>
+      </c>
+      <c r="O3" t="s">
+        <v>31</v>
+      </c>
+      <c r="P3" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L4" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4" t="s">
+        <v>48</v>
+      </c>
+      <c r="N4" t="s">
+        <v>49</v>
+      </c>
+      <c r="O4" t="s">
+        <v>31</v>
+      </c>
+      <c r="P4" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>54</v>
+      </c>
+      <c r="G5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J5" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L5" t="s">
+        <v>41</v>
+      </c>
+      <c r="M5" t="s">
+        <v>57</v>
+      </c>
+      <c r="N5" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" t="s">
+        <v>31</v>
+      </c>
+      <c r="P5" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" t="s">
+        <v>54</v>
+      </c>
+      <c r="G6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J6" t="s">
+        <v>26</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6" t="s">
+        <v>63</v>
+      </c>
+      <c r="N6" t="s">
+        <v>64</v>
+      </c>
+      <c r="O6" t="s">
+        <v>31</v>
+      </c>
+      <c r="P6" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" t="s">
+        <v>68</v>
+      </c>
+      <c r="E7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I7" t="s">
+        <v>72</v>
+      </c>
+      <c r="J7" t="s">
+        <v>26</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L7" t="s">
+        <v>62</v>
+      </c>
+      <c r="M7" t="s">
+        <v>73</v>
+      </c>
+      <c r="N7" t="s">
+        <v>74</v>
+      </c>
+      <c r="O7" t="s">
+        <v>31</v>
+      </c>
+      <c r="P7" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C8" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" t="s">
+        <v>79</v>
+      </c>
+      <c r="G8" t="s">
+        <v>80</v>
+      </c>
+      <c r="H8" t="s">
+        <v>81</v>
+      </c>
+      <c r="I8" t="s">
+        <v>82</v>
+      </c>
+      <c r="J8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" t="s">
+        <v>47</v>
+      </c>
+      <c r="M8" t="s">
+        <v>83</v>
+      </c>
+      <c r="N8" t="s">
+        <v>84</v>
+      </c>
+      <c r="O8" t="s">
+        <v>31</v>
+      </c>
+      <c r="P8" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" t="s">
+        <v>79</v>
+      </c>
+      <c r="G9" t="s">
+        <v>80</v>
+      </c>
+      <c r="H9" t="s">
+        <v>81</v>
+      </c>
+      <c r="I9" t="s">
+        <v>82</v>
+      </c>
+      <c r="J9" t="s">
+        <v>26</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" t="s">
+        <v>88</v>
+      </c>
+      <c r="M9" t="s">
+        <v>89</v>
+      </c>
+      <c r="N9" t="s">
+        <v>90</v>
+      </c>
+      <c r="O9" t="s">
+        <v>31</v>
+      </c>
+      <c r="P9" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B10" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" t="s">
+        <v>93</v>
+      </c>
+      <c r="D10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E10" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" t="s">
+        <v>79</v>
+      </c>
+      <c r="G10" t="s">
+        <v>95</v>
+      </c>
+      <c r="H10" t="s">
+        <v>38</v>
+      </c>
+      <c r="I10" t="s">
+        <v>96</v>
+      </c>
+      <c r="J10" t="s">
+        <v>26</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L10" t="s">
+        <v>97</v>
+      </c>
+      <c r="M10" t="s">
+        <v>29</v>
+      </c>
+      <c r="N10" t="s">
+        <v>98</v>
+      </c>
+      <c r="O10" t="s">
+        <v>31</v>
+      </c>
+      <c r="P10" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>